<commit_message>
Actualizacion de la documentacion
Actualizacion de la documentacion
</commit_message>
<xml_diff>
--- a/Documento/Materiales.xlsx
+++ b/Documento/Materiales.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25225"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2708d86aa79f336/Documentos/Git/Domotica-IoT/dom32-io-wifi/Documento/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="49" documentId="8_{10681902-B939-40C3-8FBC-76A8AB412AB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C253E218-BC6B-4FC5-A7BC-D950D1518EE0}"/>
+  <xr:revisionPtr revIDLastSave="84" documentId="8_{10681902-B939-40C3-8FBC-76A8AB412AB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E551EA1D-676B-4DE7-B844-574DF207462F}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="13020" xr2:uid="{40765B43-0EDD-49E3-82F7-FE87379CACB8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{40765B43-0EDD-49E3-82F7-FE87379CACB8}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Costo por placa" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="39">
   <si>
     <t>100nf / 50v</t>
   </si>
@@ -112,9 +112,6 @@
     <t>ESP-WROOM-02</t>
   </si>
   <si>
-    <t>PIC32MM0256GPM028-I-SS</t>
-  </si>
-  <si>
     <t>LM1117-3.3</t>
   </si>
   <si>
@@ -143,6 +140,18 @@
   </si>
   <si>
     <t>100uf / 25v</t>
+  </si>
+  <si>
+    <t>PIC32MM0256GPM028-I/SS (E/SS)</t>
+  </si>
+  <si>
+    <t>U$S</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>de materiales por placa</t>
   </si>
 </sst>
 </file>
@@ -178,8 +187,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -494,14 +504,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E949A11-B985-4147-9214-841059C88A3F}">
-  <dimension ref="A1:E19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -518,7 +528,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -528,12 +538,15 @@
       <c r="C2">
         <v>18</v>
       </c>
-      <c r="E2">
+      <c r="D2" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="E2" s="1">
         <f>D2*C2</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+        <v>0.54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -543,12 +556,15 @@
       <c r="C3">
         <v>1</v>
       </c>
-      <c r="E3">
+      <c r="D3" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="E3" s="1">
         <f t="shared" ref="E3:E19" si="0">D3*C3</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -558,42 +574,51 @@
       <c r="C4">
         <v>12</v>
       </c>
-      <c r="E4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D4" s="1">
+        <v>0.11</v>
+      </c>
+      <c r="E4" s="1">
+        <f t="shared" si="0"/>
+        <v>1.32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>1</v>
       </c>
       <c r="B5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0.31</v>
+      </c>
+      <c r="E5" s="1">
+        <f t="shared" si="0"/>
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
         <v>34</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6" t="s">
-        <v>35</v>
       </c>
       <c r="C6">
         <v>4</v>
       </c>
-      <c r="E6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D6" s="1">
+        <v>0.13</v>
+      </c>
+      <c r="E6" s="1">
+        <f t="shared" si="0"/>
+        <v>0.52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -603,12 +628,15 @@
       <c r="C7">
         <v>1</v>
       </c>
-      <c r="E7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D7" s="1">
+        <v>0.11</v>
+      </c>
+      <c r="E7" s="1">
+        <f t="shared" si="0"/>
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -618,12 +646,15 @@
       <c r="C8">
         <v>1</v>
       </c>
-      <c r="E8">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D8" s="1">
+        <v>0.11</v>
+      </c>
+      <c r="E8" s="1">
+        <f t="shared" si="0"/>
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -633,12 +664,15 @@
       <c r="C9">
         <v>1</v>
       </c>
-      <c r="E9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D9" s="1">
+        <v>0.11</v>
+      </c>
+      <c r="E9" s="1">
+        <f t="shared" si="0"/>
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -648,12 +682,15 @@
       <c r="C10">
         <v>3</v>
       </c>
-      <c r="E10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D10" s="1">
+        <v>0.4</v>
+      </c>
+      <c r="E10" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2000000000000002</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -663,108 +700,123 @@
       <c r="C11">
         <v>5</v>
       </c>
-      <c r="E11">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D11" s="1">
+        <v>0.08</v>
+      </c>
+      <c r="E11" s="1">
+        <f t="shared" si="0"/>
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>15</v>
       </c>
       <c r="B12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C12">
         <v>2</v>
       </c>
-      <c r="E12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D12" s="1">
+        <v>0.23</v>
+      </c>
+      <c r="E12" s="1">
+        <f t="shared" si="0"/>
+        <v>0.46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C13">
         <v>3</v>
       </c>
-      <c r="E13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D13" s="1">
+        <v>0.34</v>
+      </c>
+      <c r="E13" s="1">
+        <f t="shared" si="0"/>
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>17</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C14">
         <v>4</v>
       </c>
-      <c r="D14">
-        <v>76.78</v>
-      </c>
-      <c r="E14">
-        <f t="shared" si="0"/>
-        <v>307.12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D14" s="1">
+        <v>0.6</v>
+      </c>
+      <c r="E14" s="1">
+        <f t="shared" si="0"/>
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>21</v>
       </c>
       <c r="B15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C15">
         <v>1</v>
       </c>
-      <c r="D15">
-        <v>10.9</v>
-      </c>
-      <c r="E15">
-        <f t="shared" si="0"/>
-        <v>10.9</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D15" s="1">
+        <v>0.13</v>
+      </c>
+      <c r="E15" s="1">
+        <f t="shared" si="0"/>
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C16">
         <v>1</v>
       </c>
-      <c r="E16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D16" s="1">
+        <v>0.18</v>
+      </c>
+      <c r="E16" s="1">
+        <f t="shared" si="0"/>
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>22</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="C17">
         <v>1</v>
       </c>
-      <c r="E17">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D17" s="1">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E17" s="1">
+        <f t="shared" si="0"/>
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -774,27 +826,45 @@
       <c r="C18">
         <v>1</v>
       </c>
-      <c r="D18">
-        <v>1200</v>
-      </c>
-      <c r="E18">
-        <f t="shared" si="0"/>
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D18" s="1">
+        <v>7.2</v>
+      </c>
+      <c r="E18" s="1">
+        <f t="shared" si="0"/>
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" t="s">
         <v>28</v>
       </c>
-      <c r="B19" t="s">
-        <v>29</v>
-      </c>
       <c r="C19">
         <v>1</v>
       </c>
-      <c r="E19">
-        <f t="shared" si="0"/>
-        <v>0</v>
+      <c r="D19" s="1">
+        <v>8</v>
+      </c>
+      <c r="E19" s="1">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C25" t="s">
+        <v>37</v>
+      </c>
+      <c r="D25" t="s">
+        <v>36</v>
+      </c>
+      <c r="E25" s="1">
+        <f>SUM(E2:E24)</f>
+        <v>26.34</v>
+      </c>
+      <c r="F25" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cambio en resistencia 22R por 33R
Cambio en resistencia 22R por 33R
</commit_message>
<xml_diff>
--- a/Documento/Materiales.xlsx
+++ b/Documento/Materiales.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2708d86aa79f336/Documentos/Git/Domotica-IoT/dom32-io-wifi/Documento/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="84" documentId="8_{10681902-B939-40C3-8FBC-76A8AB412AB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E551EA1D-676B-4DE7-B844-574DF207462F}"/>
+  <xr:revisionPtr revIDLastSave="148" documentId="8_{10681902-B939-40C3-8FBC-76A8AB412AB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{427851F7-233F-4CC1-B836-118F91D54CC4}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{40765B43-0EDD-49E3-82F7-FE87379CACB8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{40765B43-0EDD-49E3-82F7-FE87379CACB8}"/>
   </bookViews>
   <sheets>
     <sheet name="Costo por placa" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="60">
   <si>
     <t>100nf / 50v</t>
   </si>
@@ -112,9 +112,6 @@
     <t>ESP-WROOM-02</t>
   </si>
   <si>
-    <t>LM1117-3.3</t>
-  </si>
-  <si>
     <t>Regulador SOT-223</t>
   </si>
   <si>
@@ -130,12 +127,6 @@
     <t>DG128-B3V</t>
   </si>
   <si>
-    <t>SRD-12VDC-SL-C</t>
-  </si>
-  <si>
-    <t>6x6x4.3 mm</t>
-  </si>
-  <si>
     <t>1000uf / 25v</t>
   </si>
   <si>
@@ -145,13 +136,85 @@
     <t>PIC32MM0256GPM028-I/SS (E/SS)</t>
   </si>
   <si>
-    <t>U$S</t>
-  </si>
-  <si>
     <t>Total</t>
   </si>
   <si>
-    <t>de materiales por placa</t>
+    <t>DigiKey</t>
+  </si>
+  <si>
+    <t>BC847C-TPCT-ND</t>
+  </si>
+  <si>
+    <t>Transistor</t>
+  </si>
+  <si>
+    <t>BC847</t>
+  </si>
+  <si>
+    <t>1965-ESP-WROOM-02D-N4CT-ND</t>
+  </si>
+  <si>
+    <t>PIC32MM0256GPM028-I/SS-ND</t>
+  </si>
+  <si>
+    <t>ZLDO1117QG33TADICT-ND</t>
+  </si>
+  <si>
+    <t>ZLDO1117</t>
+  </si>
+  <si>
+    <t>3191-M7CT-ND</t>
+  </si>
+  <si>
+    <t>3372-0805B104K500BDTR-ND</t>
+  </si>
+  <si>
+    <t>13-RC0805JR-131KLCT-ND</t>
+  </si>
+  <si>
+    <t>311-10KARCT-ND</t>
+  </si>
+  <si>
+    <t>311-33ARCT-ND</t>
+  </si>
+  <si>
+    <t>33R</t>
+  </si>
+  <si>
+    <t>LL4148-GS08CT-ND</t>
+  </si>
+  <si>
+    <t>3385-AZ943-1CH-12DE-ND</t>
+  </si>
+  <si>
+    <t>943-Series</t>
+  </si>
+  <si>
+    <t>6x6x5 mm</t>
+  </si>
+  <si>
+    <t>277-1667-ND</t>
+  </si>
+  <si>
+    <t>277-1578-ND</t>
+  </si>
+  <si>
+    <t>732-8835-1-ND</t>
+  </si>
+  <si>
+    <t>732-8630-1-ND</t>
+  </si>
+  <si>
+    <t>3147-B1701NB--20D000114U1930CT-ND</t>
+  </si>
+  <si>
+    <t>3147-B1701UY--20D000214U1930CT-ND</t>
+  </si>
+  <si>
+    <t>3147-B1701NG--20D000314U1930CT-ND</t>
+  </si>
+  <si>
+    <t>486-3458-ND</t>
   </si>
 </sst>
 </file>
@@ -496,7 +559,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -504,14 +567,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E949A11-B985-4147-9214-841059C88A3F}">
-  <dimension ref="A1:F25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F27"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.81640625" customWidth="1"/>
+    <col min="6" max="6" width="12.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -519,352 +584,469 @@
         <v>3</v>
       </c>
       <c r="C1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>13</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>18</v>
       </c>
       <c r="B2" t="s">
         <v>19</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2">
         <v>18</v>
       </c>
-      <c r="D2" s="1">
-        <v>0.03</v>
-      </c>
       <c r="E2" s="1">
-        <f>D2*C2</f>
-        <v>0.54</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.1</v>
+      </c>
+      <c r="F2" s="1">
+        <f>E2*D2</f>
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>18</v>
       </c>
       <c r="B3" t="s">
         <v>20</v>
       </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3" s="1">
-        <v>0.03</v>
+      <c r="C3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
       </c>
       <c r="E3" s="1">
-        <f t="shared" ref="E3:E19" si="0">D3*C3</f>
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.1</v>
+      </c>
+      <c r="F3" s="1">
+        <f t="shared" ref="F3:F26" si="0">E3*D3</f>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="F4" s="1"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
         <v>0</v>
       </c>
-      <c r="C4">
+      <c r="C5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5">
         <v>12</v>
       </c>
-      <c r="D4" s="1">
-        <v>0.11</v>
-      </c>
-      <c r="E4" s="1">
-        <f t="shared" si="0"/>
-        <v>1.32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5" s="1">
-        <v>0.31</v>
-      </c>
       <c r="E5" s="1">
-        <f t="shared" si="0"/>
-        <v>0.31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.05</v>
+      </c>
+      <c r="F5" s="1">
+        <f t="shared" si="0"/>
+        <v>0.60000000000000009</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C6">
+        <v>30</v>
+      </c>
+      <c r="C6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="F6" s="1">
+        <f t="shared" si="0"/>
+        <v>0.56999999999999995</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" t="s">
+        <v>55</v>
+      </c>
+      <c r="D7">
         <v>4</v>
       </c>
-      <c r="D6" s="1">
+      <c r="E7" s="1">
         <v>0.13</v>
       </c>
-      <c r="E6" s="1">
+      <c r="F7" s="1">
         <f t="shared" si="0"/>
         <v>0.52</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7">
-        <v>1</v>
-      </c>
-      <c r="D7" s="1">
-        <v>0.11</v>
-      </c>
-      <c r="E7" s="1">
-        <f t="shared" si="0"/>
-        <v>0.11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8">
-        <v>1</v>
-      </c>
-      <c r="D8" s="1">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8" s="1">
         <v>0.11</v>
       </c>
-      <c r="E8" s="1">
+      <c r="F8" s="1">
         <f t="shared" si="0"/>
         <v>0.11</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>6</v>
       </c>
       <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="F9" s="1">
+        <f t="shared" si="0"/>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" t="s">
         <v>9</v>
       </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
-      <c r="D9" s="1">
-        <v>0.11</v>
-      </c>
-      <c r="E9" s="1">
-        <f t="shared" si="0"/>
-        <v>0.11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10">
-        <v>3</v>
-      </c>
-      <c r="D10" s="1">
-        <v>0.4</v>
+      <c r="C10" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
       </c>
       <c r="E10" s="1">
-        <f t="shared" si="0"/>
-        <v>1.2000000000000002</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.1</v>
+      </c>
+      <c r="F10" s="1">
+        <f t="shared" si="0"/>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" t="s">
+        <v>42</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="F11" s="1">
+        <f t="shared" si="0"/>
+        <v>0.30000000000000004</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
         <v>12</v>
       </c>
-      <c r="C11">
+      <c r="C12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12">
         <v>5</v>
       </c>
-      <c r="D11" s="1">
-        <v>0.08</v>
-      </c>
-      <c r="E11" s="1">
-        <f t="shared" si="0"/>
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="E12" s="1">
+        <v>0.17</v>
+      </c>
+      <c r="F12" s="1">
+        <f t="shared" si="0"/>
+        <v>0.85000000000000009</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13">
+        <v>4</v>
+      </c>
+      <c r="E13" s="1">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="F13" s="1">
+        <f t="shared" si="0"/>
+        <v>0.56000000000000005</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>15</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" t="s">
+        <v>52</v>
+      </c>
+      <c r="D14">
+        <v>2</v>
+      </c>
+      <c r="E14" s="1">
+        <v>0.52</v>
+      </c>
+      <c r="F14" s="1">
+        <f t="shared" si="0"/>
+        <v>1.04</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" t="s">
         <v>29</v>
       </c>
-      <c r="C12">
-        <v>2</v>
-      </c>
-      <c r="D12" s="1">
+      <c r="C15" t="s">
+        <v>53</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+      <c r="E15" s="1">
+        <v>0.71</v>
+      </c>
+      <c r="F15" s="1">
+        <f t="shared" si="0"/>
+        <v>2.13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16">
+        <v>4</v>
+      </c>
+      <c r="E16" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="F16" s="1">
+        <f t="shared" si="0"/>
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" t="s">
+        <v>51</v>
+      </c>
+      <c r="C17" t="s">
+        <v>59</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17" s="1">
         <v>0.23</v>
       </c>
-      <c r="E12" s="1">
-        <f t="shared" si="0"/>
-        <v>0.46</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" t="s">
-        <v>30</v>
-      </c>
-      <c r="C13">
-        <v>3</v>
-      </c>
-      <c r="D13" s="1">
-        <v>0.34</v>
-      </c>
-      <c r="E13" s="1">
-        <f t="shared" si="0"/>
-        <v>1.02</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>17</v>
-      </c>
-      <c r="B14" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14">
-        <v>4</v>
-      </c>
-      <c r="D14" s="1">
-        <v>0.6</v>
-      </c>
-      <c r="E14" s="1">
-        <f t="shared" si="0"/>
-        <v>2.4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>21</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="F17" s="1">
+        <f t="shared" si="0"/>
+        <v>0.23</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" t="s">
+        <v>40</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0.67</v>
+      </c>
+      <c r="F18" s="1">
+        <f t="shared" si="0"/>
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" t="s">
         <v>32</v>
       </c>
-      <c r="C15">
-        <v>1</v>
-      </c>
-      <c r="D15" s="1">
-        <v>0.13</v>
-      </c>
-      <c r="E15" s="1">
-        <f t="shared" si="0"/>
-        <v>0.13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="C19" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19" s="1">
+        <v>2.92</v>
+      </c>
+      <c r="F19" s="1">
+        <f t="shared" si="0"/>
+        <v>2.92</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" t="s">
+        <v>38</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20" s="1">
+        <v>3.2</v>
+      </c>
+      <c r="F20" s="1">
+        <f t="shared" si="0"/>
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>26</v>
       </c>
-      <c r="B16" t="s">
-        <v>25</v>
-      </c>
-      <c r="C16">
-        <v>1</v>
-      </c>
-      <c r="D16" s="1">
-        <v>0.18</v>
-      </c>
-      <c r="E16" s="1">
-        <f t="shared" si="0"/>
-        <v>0.18</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>22</v>
-      </c>
-      <c r="B17" t="s">
-        <v>35</v>
-      </c>
-      <c r="C17">
-        <v>1</v>
-      </c>
-      <c r="D17" s="1">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="E17" s="1">
-        <f t="shared" si="0"/>
-        <v>2.2999999999999998</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>23</v>
-      </c>
-      <c r="B18" t="s">
-        <v>24</v>
-      </c>
-      <c r="C18">
-        <v>1</v>
-      </c>
-      <c r="D18" s="1">
-        <v>7.2</v>
-      </c>
-      <c r="E18" s="1">
-        <f t="shared" si="0"/>
-        <v>7.2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+      <c r="B21" t="s">
         <v>27</v>
       </c>
-      <c r="B19" t="s">
-        <v>28</v>
-      </c>
-      <c r="C19">
-        <v>1</v>
-      </c>
-      <c r="D19" s="1">
-        <v>8</v>
-      </c>
-      <c r="E19" s="1">
-        <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C25" t="s">
-        <v>37</v>
-      </c>
-      <c r="D25" t="s">
-        <v>36</v>
-      </c>
-      <c r="E25" s="1">
-        <f>SUM(E2:E24)</f>
-        <v>26.34</v>
-      </c>
-      <c r="F25" t="s">
-        <v>38</v>
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21" s="1">
+        <v>7.4</v>
+      </c>
+      <c r="F21" s="1">
+        <f t="shared" si="0"/>
+        <v>7.4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="F22" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="F23" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="F24" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="F25" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="F26" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="D27" t="s">
+        <v>33</v>
+      </c>
+      <c r="F27" s="1">
+        <f>SUM(F2:F26)</f>
+        <v>25.800000000000004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>